<commit_message>
Excel downloads: keep formulas, links, dropdowns and conditional formats; clear only price values (header-aware, fixes Dammam quantity column)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGLiEJkpTWKADYGLjZmT4M
</commit_message>
<xml_diff>
--- a/assets/docs/boq-dammam.xlsx
+++ b/assets/docs/boq-dammam.xlsx
@@ -3136,7 +3136,9 @@
         <v>23</v>
       </c>
       <c r="F3" s="36"/>
-      <c r="G3" s="37"/>
+      <c r="G3" s="37">
+        <f t="shared" ref="G3:G6" si="1">D3*F3</f>
+      </c>
       <c r="H3" s="38"/>
       <c r="I3" s="39"/>
       <c r="J3" s="39"/>
@@ -3176,7 +3178,9 @@
         <v>23</v>
       </c>
       <c r="F4" s="45"/>
-      <c r="G4" s="46"/>
+      <c r="G4" s="46">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H4" s="48"/>
       <c r="I4" s="39"/>
       <c r="J4" s="39"/>
@@ -3216,7 +3220,9 @@
         <v>23</v>
       </c>
       <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="G5" s="46">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H5" s="48"/>
       <c r="I5" s="39"/>
       <c r="J5" s="39"/>
@@ -3256,7 +3262,9 @@
         <v>23</v>
       </c>
       <c r="F6" s="45"/>
-      <c r="G6" s="46"/>
+      <c r="G6" s="46">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H6" s="48"/>
       <c r="I6" s="39"/>
       <c r="J6" s="39"/>
@@ -3288,7 +3296,9 @@
       <c r="D7" s="69"/>
       <c r="E7" s="67"/>
       <c r="F7" s="70"/>
-      <c r="G7" s="70"/>
+      <c r="G7" s="70">
+        <f>SUM(G3:G6)</f>
+      </c>
       <c r="H7" s="71"/>
       <c r="I7" s="72"/>
       <c r="J7" s="72"/>
@@ -3362,7 +3372,9 @@
         <v>29</v>
       </c>
       <c r="F9" s="63"/>
-      <c r="G9" s="58"/>
+      <c r="G9" s="58">
+        <f>D9*F9</f>
+      </c>
       <c r="H9" s="80"/>
       <c r="I9" s="72"/>
       <c r="J9" s="72"/>
@@ -3394,7 +3406,9 @@
       <c r="D10" s="67"/>
       <c r="E10" s="67"/>
       <c r="F10" s="70"/>
-      <c r="G10" s="70"/>
+      <c r="G10" s="70">
+        <f>SUM(G9)</f>
+      </c>
       <c r="H10" s="71"/>
       <c r="I10" s="72"/>
       <c r="J10" s="72"/>
@@ -3468,7 +3482,9 @@
         <v>47</v>
       </c>
       <c r="F12" s="45"/>
-      <c r="G12" s="46"/>
+      <c r="G12" s="46">
+        <f t="shared" ref="G12:G13" si="2">D12*F12</f>
+      </c>
       <c r="H12" s="48"/>
       <c r="I12" s="72"/>
       <c r="J12" s="72"/>
@@ -3508,7 +3524,9 @@
         <v>53</v>
       </c>
       <c r="F13" s="45"/>
-      <c r="G13" s="46"/>
+      <c r="G13" s="46">
+        <f t="shared" si="2"/>
+      </c>
       <c r="H13" s="48"/>
       <c r="I13" s="72"/>
       <c r="J13" s="72"/>
@@ -3540,7 +3558,9 @@
       <c r="D14" s="69"/>
       <c r="E14" s="67"/>
       <c r="F14" s="70"/>
-      <c r="G14" s="70"/>
+      <c r="G14" s="70">
+        <f>SUM(G12:G13)</f>
+      </c>
       <c r="H14" s="71"/>
       <c r="I14" s="72"/>
       <c r="J14" s="72"/>
@@ -3614,7 +3634,9 @@
         <v>23</v>
       </c>
       <c r="F16" s="95"/>
-      <c r="G16" s="96"/>
+      <c r="G16" s="96">
+        <f>D16*F16</f>
+      </c>
       <c r="H16" s="97"/>
       <c r="I16" s="29"/>
       <c r="J16" s="29"/>
@@ -3676,7 +3698,9 @@
       <c r="D18" s="69"/>
       <c r="E18" s="67"/>
       <c r="F18" s="70"/>
-      <c r="G18" s="70"/>
+      <c r="G18" s="70">
+        <f>G16</f>
+      </c>
       <c r="H18" s="71"/>
       <c r="I18" s="72"/>
       <c r="J18" s="72"/>
@@ -3750,7 +3774,9 @@
         <v>47</v>
       </c>
       <c r="F20" s="108"/>
-      <c r="G20" s="109"/>
+      <c r="G20" s="109">
+        <f t="shared" ref="G20:G21" si="3">D20*F20</f>
+      </c>
       <c r="H20" s="80" t="e">
         <v>#VALUE!</v>
       </c>
@@ -3772,7 +3798,9 @@
         <v>47</v>
       </c>
       <c r="F21" s="108"/>
-      <c r="G21" s="109"/>
+      <c r="G21" s="109">
+        <f t="shared" si="3"/>
+      </c>
       <c r="H21" s="80" t="e">
         <v>#VALUE!</v>
       </c>
@@ -3786,7 +3814,9 @@
       <c r="D22" s="69"/>
       <c r="E22" s="67"/>
       <c r="F22" s="70"/>
-      <c r="G22" s="70"/>
+      <c r="G22" s="70">
+        <f>SUM(G20:G21)</f>
+      </c>
       <c r="H22" s="71"/>
       <c r="I22" s="72"/>
       <c r="J22" s="72"/>
@@ -3818,7 +3848,9 @@
       <c r="D23" s="113"/>
       <c r="E23" s="111"/>
       <c r="F23" s="111"/>
-      <c r="G23" s="114"/>
+      <c r="G23" s="114">
+        <f>G7+G10+G14+G18+G22</f>
+      </c>
       <c r="H23" s="110"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -10772,7 +10804,9 @@
         <v>29</v>
       </c>
       <c r="F3" s="54"/>
-      <c r="G3" s="57"/>
+      <c r="G3" s="57">
+        <f t="shared" ref="G3:G18" si="1">D3*F3</f>
+      </c>
       <c r="H3" s="59" t="e">
         <v>#VALUE!</v>
       </c>
@@ -10794,7 +10828,9 @@
         <v>29</v>
       </c>
       <c r="F4" s="63"/>
-      <c r="G4" s="57"/>
+      <c r="G4" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H4" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -10816,7 +10852,9 @@
         <v>29</v>
       </c>
       <c r="F5" s="63"/>
-      <c r="G5" s="57"/>
+      <c r="G5" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H5" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -10838,7 +10876,9 @@
         <v>29</v>
       </c>
       <c r="F6" s="121"/>
-      <c r="G6" s="57"/>
+      <c r="G6" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H6" s="123"/>
     </row>
     <row r="7" ht="231.75" customHeight="1">
@@ -10858,7 +10898,9 @@
         <v>29</v>
       </c>
       <c r="F7" s="63"/>
-      <c r="G7" s="57"/>
+      <c r="G7" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H7" s="64"/>
     </row>
     <row r="8" ht="231.75" customHeight="1">
@@ -10878,7 +10920,9 @@
         <v>29</v>
       </c>
       <c r="F8" s="87"/>
-      <c r="G8" s="57"/>
+      <c r="G8" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H8" s="124"/>
       <c r="J8" s="88"/>
       <c r="K8" s="89"/>
@@ -10914,7 +10958,9 @@
         <v>29</v>
       </c>
       <c r="F9" s="128"/>
-      <c r="G9" s="57"/>
+      <c r="G9" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H9" s="129" t="e">
         <v>#VALUE!</v>
       </c>
@@ -10956,7 +11002,9 @@
         <v>29</v>
       </c>
       <c r="F10" s="63"/>
-      <c r="G10" s="57"/>
+      <c r="G10" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H10" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -10998,7 +11046,9 @@
         <v>29</v>
       </c>
       <c r="F11" s="63"/>
-      <c r="G11" s="57"/>
+      <c r="G11" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H11" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11020,7 +11070,9 @@
         <v>29</v>
       </c>
       <c r="F12" s="133"/>
-      <c r="G12" s="57"/>
+      <c r="G12" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H12" s="135" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11042,7 +11094,9 @@
         <v>29</v>
       </c>
       <c r="F13" s="87"/>
-      <c r="G13" s="57"/>
+      <c r="G13" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H13" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11080,7 +11134,9 @@
         <v>29</v>
       </c>
       <c r="F14" s="142"/>
-      <c r="G14" s="57"/>
+      <c r="G14" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H14" s="143" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11118,7 +11174,9 @@
         <v>29</v>
       </c>
       <c r="F15" s="87"/>
-      <c r="G15" s="57"/>
+      <c r="G15" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H15" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11156,7 +11214,9 @@
         <v>29</v>
       </c>
       <c r="F16" s="87"/>
-      <c r="G16" s="57"/>
+      <c r="G16" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H16" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11194,7 +11254,9 @@
         <v>47</v>
       </c>
       <c r="F17" s="87"/>
-      <c r="G17" s="57"/>
+      <c r="G17" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H17" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11232,7 +11294,9 @@
         <v>45</v>
       </c>
       <c r="F18" s="63"/>
-      <c r="G18" s="57"/>
+      <c r="G18" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H18" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11246,7 +11310,9 @@
       <c r="D19" s="148"/>
       <c r="E19" s="144"/>
       <c r="F19" s="149"/>
-      <c r="G19" s="149"/>
+      <c r="G19" s="149">
+        <f>SUM(G3:G18)</f>
+      </c>
       <c r="H19" s="150"/>
       <c r="I19" s="72"/>
       <c r="J19" s="72"/>
@@ -11320,7 +11386,9 @@
         <v>29</v>
       </c>
       <c r="F21" s="63"/>
-      <c r="G21" s="58"/>
+      <c r="G21" s="58">
+        <f t="shared" ref="G21:G24" si="2">D21*F21</f>
+      </c>
       <c r="H21" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11362,7 +11430,9 @@
         <v>29</v>
       </c>
       <c r="F22" s="63"/>
-      <c r="G22" s="58"/>
+      <c r="G22" s="58">
+        <f t="shared" si="2"/>
+      </c>
       <c r="H22" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11404,7 +11474,9 @@
         <v>29</v>
       </c>
       <c r="F23" s="63"/>
-      <c r="G23" s="58"/>
+      <c r="G23" s="58">
+        <f t="shared" si="2"/>
+      </c>
       <c r="H23" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11446,7 +11518,9 @@
         <v>29</v>
       </c>
       <c r="F24" s="54"/>
-      <c r="G24" s="58"/>
+      <c r="G24" s="58">
+        <f t="shared" si="2"/>
+      </c>
       <c r="H24" s="135" t="e">
         <v>#VALUE!</v>
       </c>
@@ -11480,7 +11554,9 @@
       <c r="D25" s="157"/>
       <c r="E25" s="153"/>
       <c r="F25" s="158"/>
-      <c r="G25" s="158"/>
+      <c r="G25" s="158">
+        <f>SUM(G21:G24)</f>
+      </c>
       <c r="H25" s="159"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -11492,7 +11568,9 @@
       <c r="D26" s="103"/>
       <c r="E26" s="101"/>
       <c r="F26" s="101"/>
-      <c r="G26" s="104"/>
+      <c r="G26" s="104">
+        <f>G19+G25</f>
+      </c>
       <c r="H26" s="101"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -15501,17 +15579,16 @@
       <c r="D3" s="53">
         <v>7.0</v>
       </c>
-      <c r="E3" s="53">
-        <v>2070.0</v>
-      </c>
-      <c r="F3" s="51"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="51">
+        <v>21.0</v>
+      </c>
       <c r="G3" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H3" s="56"/>
       <c r="I3" s="58">
         <f t="shared" ref="I3:I6" si="1">F3*H3</f>
-        <v>0</v>
       </c>
       <c r="J3" s="60" t="e">
         <v>#VALUE!</v>
@@ -15550,17 +15627,16 @@
       <c r="D4" s="53">
         <v>7.0</v>
       </c>
-      <c r="E4" s="53">
-        <v>2070.0</v>
-      </c>
-      <c r="F4" s="51"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="51">
+        <v>1.0</v>
+      </c>
       <c r="G4" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H4" s="63"/>
       <c r="I4" s="58">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="J4" s="64" t="e">
         <v>#VALUE!</v>
@@ -15599,17 +15675,16 @@
       <c r="D5" s="53">
         <v>11.0</v>
       </c>
-      <c r="E5" s="53">
-        <v>2070.0</v>
-      </c>
-      <c r="F5" s="51"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="51">
+        <v>1.0</v>
+      </c>
       <c r="G5" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H5" s="63"/>
       <c r="I5" s="58">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="J5" s="64" t="e">
         <v>#VALUE!</v>
@@ -15648,17 +15723,16 @@
       <c r="D6" s="122">
         <v>3.0</v>
       </c>
-      <c r="E6" s="122">
-        <v>2070.0</v>
-      </c>
-      <c r="F6" s="51"/>
+      <c r="E6" s="122"/>
+      <c r="F6" s="51">
+        <v>3.0</v>
+      </c>
       <c r="G6" s="52" t="s">
         <v>47</v>
       </c>
       <c r="H6" s="54"/>
       <c r="I6" s="57">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="J6" s="57" t="e">
         <v>#VALUE!</v>
@@ -15677,7 +15751,6 @@
       <c r="H7" s="70"/>
       <c r="I7" s="70">
         <f>SUM(I3:I6)</f>
-        <v>0</v>
       </c>
       <c r="J7" s="70"/>
     </row>
@@ -15730,17 +15803,16 @@
       <c r="D9" s="53">
         <v>1.0</v>
       </c>
-      <c r="E9" s="53">
-        <v>1090.0</v>
-      </c>
-      <c r="F9" s="51"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="51">
+        <v>133.0</v>
+      </c>
       <c r="G9" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H9" s="63"/>
       <c r="I9" s="58">
         <f t="shared" ref="I9:I15" si="2">F9*H9</f>
-        <v>0</v>
       </c>
       <c r="J9" s="58" t="e">
         <v>#VALUE!</v>
@@ -15759,17 +15831,16 @@
       <c r="D10" s="122">
         <v>2.0</v>
       </c>
-      <c r="E10" s="122">
-        <v>2170.0</v>
-      </c>
-      <c r="F10" s="51"/>
+      <c r="E10" s="122"/>
+      <c r="F10" s="51">
+        <v>4.0</v>
+      </c>
       <c r="G10" s="52" t="s">
         <v>29</v>
       </c>
       <c r="H10" s="54"/>
       <c r="I10" s="57">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J10" s="135" t="e">
         <v>#VALUE!</v>
@@ -15808,17 +15879,16 @@
       <c r="D11" s="122">
         <v>3.0</v>
       </c>
-      <c r="E11" s="122">
-        <v>2170.0</v>
-      </c>
-      <c r="F11" s="51"/>
+      <c r="E11" s="122"/>
+      <c r="F11" s="51">
+        <v>8.0</v>
+      </c>
       <c r="G11" s="52" t="s">
         <v>29</v>
       </c>
       <c r="H11" s="54"/>
       <c r="I11" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J11" s="135" t="e">
         <v>#VALUE!</v>
@@ -15857,17 +15927,16 @@
       <c r="D12" s="53">
         <v>6.0</v>
       </c>
-      <c r="E12" s="53">
-        <v>2170.0</v>
-      </c>
-      <c r="F12" s="51"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="51">
+        <v>1.0</v>
+      </c>
       <c r="G12" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H12" s="63"/>
       <c r="I12" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J12" s="64"/>
     </row>
@@ -15884,17 +15953,16 @@
       <c r="D13" s="53">
         <v>12.0</v>
       </c>
-      <c r="E13" s="53">
-        <v>2170.0</v>
-      </c>
-      <c r="F13" s="51"/>
+      <c r="E13" s="53"/>
+      <c r="F13" s="51">
+        <v>1.0</v>
+      </c>
       <c r="G13" s="146" t="s">
         <v>29</v>
       </c>
       <c r="H13" s="87"/>
       <c r="I13" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J13" s="84"/>
       <c r="L13" s="88"/>
@@ -15927,17 +15995,16 @@
       <c r="D14" s="53">
         <v>7.0</v>
       </c>
-      <c r="E14" s="53">
-        <v>2170.0</v>
-      </c>
-      <c r="F14" s="51"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="51">
+        <v>2.0</v>
+      </c>
       <c r="G14" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H14" s="63"/>
       <c r="I14" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J14" s="64"/>
     </row>
@@ -15954,17 +16021,16 @@
       <c r="D15" s="53">
         <v>1.0</v>
       </c>
-      <c r="E15" s="53">
-        <v>780.0</v>
-      </c>
-      <c r="F15" s="51"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="51">
+        <v>19.0</v>
+      </c>
       <c r="G15" s="55" t="s">
         <v>29</v>
       </c>
       <c r="H15" s="63"/>
       <c r="I15" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
       </c>
       <c r="J15" s="58" t="e">
         <v>#VALUE!</v>
@@ -15983,7 +16049,6 @@
       <c r="H16" s="70"/>
       <c r="I16" s="70">
         <f>SUM(I9:I15)</f>
-        <v>0</v>
       </c>
       <c r="J16" s="70"/>
     </row>
@@ -16000,7 +16065,6 @@
       <c r="H17" s="101"/>
       <c r="I17" s="104">
         <f>I7+I16</f>
-        <v>0</v>
       </c>
       <c r="J17" s="104"/>
     </row>
@@ -21022,7 +21086,9 @@
         <v>29</v>
       </c>
       <c r="F3" s="54"/>
-      <c r="G3" s="57"/>
+      <c r="G3" s="57">
+        <f t="shared" ref="G3:G12" si="1">D3*F3</f>
+      </c>
       <c r="H3" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21044,7 +21110,9 @@
         <v>29</v>
       </c>
       <c r="F4" s="54"/>
-      <c r="G4" s="57"/>
+      <c r="G4" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H4" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21066,7 +21134,9 @@
         <v>45</v>
       </c>
       <c r="F5" s="63"/>
-      <c r="G5" s="58"/>
+      <c r="G5" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H5" s="58" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21088,7 +21158,9 @@
         <v>47</v>
       </c>
       <c r="F6" s="63"/>
-      <c r="G6" s="58"/>
+      <c r="G6" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H6" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21110,7 +21182,9 @@
         <v>29</v>
       </c>
       <c r="F7" s="63"/>
-      <c r="G7" s="58"/>
+      <c r="G7" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H7" s="85"/>
     </row>
     <row r="8" ht="90.0" customHeight="1">
@@ -21130,7 +21204,9 @@
         <v>29</v>
       </c>
       <c r="F8" s="63"/>
-      <c r="G8" s="57"/>
+      <c r="G8" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H8" s="85"/>
     </row>
     <row r="9" ht="152.25" customHeight="1">
@@ -21150,7 +21226,9 @@
         <v>29</v>
       </c>
       <c r="F9" s="87"/>
-      <c r="G9" s="58"/>
+      <c r="G9" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H9" s="84" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21188,7 +21266,9 @@
         <v>47</v>
       </c>
       <c r="F10" s="63"/>
-      <c r="G10" s="58"/>
+      <c r="G10" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H10" s="58" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21210,7 +21290,9 @@
         <v>29</v>
       </c>
       <c r="F11" s="54"/>
-      <c r="G11" s="57"/>
+      <c r="G11" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H11" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21232,7 +21314,9 @@
         <v>29</v>
       </c>
       <c r="F12" s="63"/>
-      <c r="G12" s="58"/>
+      <c r="G12" s="58">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H12" s="64" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21246,7 +21330,9 @@
       <c r="D13" s="69"/>
       <c r="E13" s="67"/>
       <c r="F13" s="70"/>
-      <c r="G13" s="70"/>
+      <c r="G13" s="70">
+        <f>SUM(G3:G12)</f>
+      </c>
       <c r="H13" s="70"/>
     </row>
     <row r="14">
@@ -21300,7 +21386,9 @@
         <v>45</v>
       </c>
       <c r="F15" s="63"/>
-      <c r="G15" s="58"/>
+      <c r="G15" s="58">
+        <f>D15*F15</f>
+      </c>
       <c r="H15" s="58" t="e">
         <v>#VALUE!</v>
       </c>
@@ -21314,7 +21402,9 @@
       <c r="D16" s="69"/>
       <c r="E16" s="67"/>
       <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
+      <c r="G16" s="70">
+        <f>G15</f>
+      </c>
       <c r="H16" s="70"/>
     </row>
     <row r="17">
@@ -21326,7 +21416,9 @@
       <c r="D17" s="103"/>
       <c r="E17" s="101"/>
       <c r="F17" s="101"/>
-      <c r="G17" s="104"/>
+      <c r="G17" s="104">
+        <f>G13+G16</f>
+      </c>
       <c r="H17" s="104"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -25362,7 +25454,9 @@
         <v>45</v>
       </c>
       <c r="F3" s="63"/>
-      <c r="G3" s="58" t="str"/>
+      <c r="G3" s="58" t="str">
+        <f>G2</f>
+      </c>
       <c r="H3" s="58" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25404,7 +25498,9 @@
         <v>45</v>
       </c>
       <c r="F4" s="166"/>
-      <c r="G4" s="58"/>
+      <c r="G4" s="58">
+        <f>D4*F4</f>
+      </c>
       <c r="H4" s="167" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25434,7 +25530,9 @@
       <c r="D5" s="69"/>
       <c r="E5" s="67"/>
       <c r="F5" s="70"/>
-      <c r="G5" s="70"/>
+      <c r="G5" s="70">
+        <f>SUM(G3:G4)</f>
+      </c>
       <c r="H5" s="70"/>
     </row>
     <row r="6">
@@ -25488,7 +25586,9 @@
         <v>29</v>
       </c>
       <c r="F7" s="54"/>
-      <c r="G7" s="57"/>
+      <c r="G7" s="57">
+        <f t="shared" ref="G7:G8" si="1">D7*F7</f>
+      </c>
       <c r="H7" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25510,7 +25610,9 @@
         <v>29</v>
       </c>
       <c r="F8" s="54"/>
-      <c r="G8" s="57"/>
+      <c r="G8" s="57">
+        <f t="shared" si="1"/>
+      </c>
       <c r="H8" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25524,7 +25626,9 @@
       <c r="D9" s="69"/>
       <c r="E9" s="67"/>
       <c r="F9" s="70"/>
-      <c r="G9" s="70"/>
+      <c r="G9" s="70">
+        <f>SUM(G7:G8)</f>
+      </c>
       <c r="H9" s="70"/>
     </row>
     <row r="10">
@@ -25578,7 +25682,9 @@
         <v>29</v>
       </c>
       <c r="F11" s="54"/>
-      <c r="G11" s="57"/>
+      <c r="G11" s="57">
+        <f>D11*F11</f>
+      </c>
       <c r="H11" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25592,7 +25698,9 @@
       <c r="D12" s="69"/>
       <c r="E12" s="67"/>
       <c r="F12" s="70"/>
-      <c r="G12" s="70"/>
+      <c r="G12" s="70">
+        <f>SUM(G10:G11)</f>
+      </c>
       <c r="H12" s="70"/>
     </row>
     <row r="13">
@@ -25646,7 +25754,9 @@
         <v>29</v>
       </c>
       <c r="F14" s="54"/>
-      <c r="G14" s="57"/>
+      <c r="G14" s="57">
+        <f>D14*F14</f>
+      </c>
       <c r="H14" s="57" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25680,7 +25790,9 @@
       <c r="D15" s="69"/>
       <c r="E15" s="67"/>
       <c r="F15" s="70"/>
-      <c r="G15" s="70"/>
+      <c r="G15" s="70">
+        <f>SUM(G13:G14)</f>
+      </c>
       <c r="H15" s="70"/>
     </row>
     <row r="16">
@@ -25734,7 +25846,9 @@
         <v>29</v>
       </c>
       <c r="F17" s="63"/>
-      <c r="G17" s="58"/>
+      <c r="G17" s="58">
+        <f>D17*F17</f>
+      </c>
       <c r="H17" s="58" t="e">
         <v>#VALUE!</v>
       </c>
@@ -25748,7 +25862,9 @@
       <c r="D18" s="69"/>
       <c r="E18" s="67"/>
       <c r="F18" s="70"/>
-      <c r="G18" s="70"/>
+      <c r="G18" s="70">
+        <f>SUM(G17)</f>
+      </c>
       <c r="H18" s="70"/>
     </row>
     <row r="19">
@@ -25760,7 +25876,9 @@
       <c r="D19" s="103"/>
       <c r="E19" s="101"/>
       <c r="F19" s="101"/>
-      <c r="G19" s="104"/>
+      <c r="G19" s="104">
+        <f>G5+G9+G12+G15+G18</f>
+      </c>
       <c r="H19" s="101"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">

</xml_diff>